<commit_message>
Add PiN results (Excel) for Mozambique___MOZ
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Mozambique___MOZ/PiN_results_Mozambique___MOZ_0930_01PM.xlsx
+++ b/platform_PiN_output/Mozambique___MOZ/PiN_results_Mozambique___MOZ_0930_01PM.xlsx
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>303889</v>
+        <v>255147</v>
       </c>
       <c r="F6" s="9" t="n"/>
       <c r="G6" s="9" t="n"/>
@@ -772,34 +772,34 @@
         <v>1391945</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>78.2</v>
+        <v>81.7</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>1088056</v>
+        <v>1136798</v>
       </c>
       <c r="M6" s="8" t="n">
-        <v>20.7</v>
+        <v>16.5</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>288695</v>
+        <v>230327</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>0.5</v>
+        <v>1.3</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>7647</v>
+        <v>18005</v>
       </c>
       <c r="Q6" s="8" t="n">
         <v>0.5</v>
       </c>
       <c r="R6" s="8" t="n">
-        <v>7547</v>
+        <v>6815</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>21.8</v>
+        <v>18.3</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>303889</v>
+        <v>255147</v>
       </c>
     </row>
     <row r="7">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>201915</v>
+        <v>178734</v>
       </c>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
@@ -834,34 +834,34 @@
         <v>991607</v>
       </c>
       <c r="K7" s="10" t="n">
-        <v>79.59999999999999</v>
+        <v>82</v>
       </c>
       <c r="L7" s="10" t="n">
-        <v>789692</v>
+        <v>812873</v>
       </c>
       <c r="M7" s="10" t="n">
-        <v>19.7</v>
+        <v>16.8</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>195609</v>
+        <v>166400</v>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="P7" s="10" t="n">
-        <v>4283</v>
+        <v>10056</v>
       </c>
       <c r="Q7" s="10" t="n">
         <v>0.2</v>
       </c>
       <c r="R7" s="10" t="n">
-        <v>2023</v>
+        <v>2278</v>
       </c>
       <c r="S7" s="10" t="n">
-        <v>20.4</v>
+        <v>18</v>
       </c>
       <c r="T7" s="10" t="n">
-        <v>201915</v>
+        <v>178734</v>
       </c>
     </row>
     <row r="8">
@@ -878,7 +878,7 @@
         </is>
       </c>
       <c r="E8" s="10" t="n">
-        <v>43197</v>
+        <v>34710</v>
       </c>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
@@ -896,34 +896,34 @@
         <v>156856</v>
       </c>
       <c r="K8" s="10" t="n">
-        <v>72.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="L8" s="10" t="n">
-        <v>113659</v>
+        <v>122146</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>24.8</v>
+        <v>17.9</v>
       </c>
       <c r="N8" s="10" t="n">
-        <v>38897</v>
+        <v>28028</v>
       </c>
       <c r="O8" s="10" t="n">
-        <v>0.7</v>
+        <v>2.3</v>
       </c>
       <c r="P8" s="10" t="n">
-        <v>1038</v>
+        <v>3678</v>
       </c>
       <c r="Q8" s="10" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="R8" s="10" t="n">
-        <v>3262</v>
+        <v>3004</v>
       </c>
       <c r="S8" s="10" t="n">
-        <v>27.5</v>
+        <v>22.1</v>
       </c>
       <c r="T8" s="10" t="n">
-        <v>43197</v>
+        <v>34710</v>
       </c>
     </row>
     <row r="9">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>58778</v>
+        <v>41704</v>
       </c>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
@@ -958,34 +958,34 @@
         <v>243482</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>75.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>184704</v>
+        <v>201778</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>22.3</v>
+        <v>14.7</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>54189</v>
+        <v>35899</v>
       </c>
       <c r="O9" s="10" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="P9" s="10" t="n">
-        <v>2327</v>
+        <v>4271</v>
       </c>
       <c r="Q9" s="10" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="R9" s="10" t="n">
-        <v>2262</v>
+        <v>1533</v>
       </c>
       <c r="S9" s="10" t="n">
-        <v>24.1</v>
+        <v>17.1</v>
       </c>
       <c r="T9" s="10" t="n">
-        <v>58778</v>
+        <v>41704</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>149396</v>
+        <v>125471</v>
       </c>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>154493</v>
+        <v>129676</v>
       </c>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>30679</v>
+        <v>25833</v>
       </c>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="E13" s="12" t="n">
-        <v>30389</v>
+        <v>25515</v>
       </c>
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
@@ -1243,22 +1243,22 @@
         <v>11474</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>66.5</v>
+        <v>70.5</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>7630</v>
+        <v>8087</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>33.4</v>
+        <v>24.5</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>3830</v>
+        <v>2814</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="L6" s="24" t="n">
-        <v>14</v>
+        <v>572</v>
       </c>
       <c r="M6" s="25" t="n">
         <v>0</v>
@@ -1267,10 +1267,10 @@
         <v>0</v>
       </c>
       <c r="O6" s="26" t="n">
-        <v>33.5</v>
+        <v>29.5</v>
       </c>
       <c r="P6" s="26" t="n">
-        <v>3844</v>
+        <v>3387</v>
       </c>
       <c r="Q6" s="27" t="inlineStr">
         <is>
@@ -1292,22 +1292,22 @@
         <v>109979</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>94.09999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>103527</v>
+        <v>105994</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>5.9</v>
+        <v>3.2</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>6452</v>
+        <v>3502</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="L7" s="24" t="n">
-        <v>0</v>
+        <v>484</v>
       </c>
       <c r="M7" s="25" t="n">
         <v>0</v>
@@ -1316,10 +1316,10 @@
         <v>0</v>
       </c>
       <c r="O7" s="26" t="n">
-        <v>5.9</v>
+        <v>3.6</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>6452</v>
+        <v>3985</v>
       </c>
       <c r="Q7" s="27" t="inlineStr">
         <is>
@@ -1341,38 +1341,38 @@
         <v>74486</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>79.09999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>58941</v>
+        <v>60790</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>16.8</v>
+        <v>14.8</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>12541</v>
+        <v>11052</v>
       </c>
       <c r="K8" s="24" t="n">
         <v>0.1</v>
       </c>
       <c r="L8" s="24" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="M8" s="25" t="n">
-        <v>3.9</v>
+        <v>3.4</v>
       </c>
       <c r="N8" s="25" t="n">
-        <v>2915</v>
+        <v>2545</v>
       </c>
       <c r="O8" s="26" t="n">
-        <v>20.9</v>
+        <v>18.4</v>
       </c>
       <c r="P8" s="26" t="n">
-        <v>15545</v>
+        <v>13696</v>
       </c>
       <c r="Q8" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -1390,34 +1390,34 @@
         <v>71470</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>85.5</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>61127</v>
+        <v>61043</v>
       </c>
       <c r="I9" s="23" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="J9" s="23" t="n">
-        <v>10082</v>
+        <v>10113</v>
       </c>
       <c r="K9" s="24" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="24" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="M9" s="25" t="n">
         <v>0.4</v>
       </c>
       <c r="N9" s="25" t="n">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="O9" s="26" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="P9" s="26" t="n">
-        <v>10343</v>
+        <v>10427</v>
       </c>
       <c r="Q9" s="27" t="inlineStr">
         <is>
@@ -1439,22 +1439,22 @@
         <v>122911</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>80.59999999999999</v>
+        <v>85.7</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>99123</v>
+        <v>105290</v>
       </c>
       <c r="I10" s="23" t="n">
-        <v>18.1</v>
+        <v>13.8</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>22212</v>
+        <v>16990</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>1.3</v>
+        <v>0.5</v>
       </c>
       <c r="L10" s="24" t="n">
-        <v>1576</v>
+        <v>631</v>
       </c>
       <c r="M10" s="25" t="n">
         <v>0</v>
@@ -1463,10 +1463,10 @@
         <v>0</v>
       </c>
       <c r="O10" s="26" t="n">
-        <v>19.4</v>
+        <v>14.3</v>
       </c>
       <c r="P10" s="26" t="n">
-        <v>23788</v>
+        <v>17621</v>
       </c>
       <c r="Q10" s="27" t="inlineStr">
         <is>
@@ -1488,16 +1488,16 @@
         <v>11345</v>
       </c>
       <c r="G11" s="22" t="n">
-        <v>96.8</v>
+        <v>97.7</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>10984</v>
+        <v>11087</v>
       </c>
       <c r="I11" s="23" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>327</v>
+        <v>216</v>
       </c>
       <c r="K11" s="24" t="n">
         <v>0</v>
@@ -1506,16 +1506,16 @@
         <v>0</v>
       </c>
       <c r="M11" s="25" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="N11" s="25" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="O11" s="26" t="n">
-        <v>3.2</v>
+        <v>2.3</v>
       </c>
       <c r="P11" s="26" t="n">
-        <v>361</v>
+        <v>258</v>
       </c>
       <c r="Q11" s="27" t="inlineStr">
         <is>
@@ -1537,34 +1537,34 @@
         <v>63498</v>
       </c>
       <c r="G12" s="22" t="n">
-        <v>68.09999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>43225</v>
+        <v>47968</v>
       </c>
       <c r="I12" s="23" t="n">
-        <v>30.7</v>
+        <v>20.2</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>19523</v>
+        <v>12847</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>0.5</v>
+        <v>3.6</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>290</v>
+        <v>2264</v>
       </c>
       <c r="M12" s="25" t="n">
         <v>0.7</v>
       </c>
       <c r="N12" s="25" t="n">
-        <v>460</v>
+        <v>419</v>
       </c>
       <c r="O12" s="26" t="n">
-        <v>31.9</v>
+        <v>24.5</v>
       </c>
       <c r="P12" s="26" t="n">
-        <v>20273</v>
+        <v>15530</v>
       </c>
       <c r="Q12" s="27" t="inlineStr">
         <is>
@@ -1586,22 +1586,22 @@
         <v>32018</v>
       </c>
       <c r="G13" s="22" t="n">
-        <v>68.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>22045</v>
+        <v>23104</v>
       </c>
       <c r="I13" s="23" t="n">
-        <v>31.1</v>
+        <v>12.3</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>9973</v>
+        <v>3925</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0</v>
+        <v>15.6</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0</v>
+        <v>4988</v>
       </c>
       <c r="M13" s="25" t="n">
         <v>0</v>
@@ -1610,10 +1610,10 @@
         <v>0</v>
       </c>
       <c r="O13" s="26" t="n">
-        <v>31.1</v>
+        <v>27.8</v>
       </c>
       <c r="P13" s="26" t="n">
-        <v>9973</v>
+        <v>8914</v>
       </c>
       <c r="Q13" s="27" t="inlineStr">
         <is>
@@ -1635,34 +1635,34 @@
         <v>16937</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>56.1</v>
+        <v>54.3</v>
       </c>
       <c r="H14" s="22" t="n">
-        <v>9497</v>
+        <v>9191</v>
       </c>
       <c r="I14" s="23" t="n">
-        <v>43.7</v>
+        <v>45.6</v>
       </c>
       <c r="J14" s="23" t="n">
-        <v>7405</v>
+        <v>7723</v>
       </c>
       <c r="K14" s="24" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M14" s="25" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="N14" s="25" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="O14" s="26" t="n">
-        <v>43.9</v>
+        <v>45.7</v>
       </c>
       <c r="P14" s="26" t="n">
-        <v>7440</v>
+        <v>7746</v>
       </c>
       <c r="Q14" s="27" t="inlineStr">
         <is>
@@ -1684,38 +1684,38 @@
         <v>60289</v>
       </c>
       <c r="G15" s="22" t="n">
-        <v>70.3</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="H15" s="22" t="n">
-        <v>42372</v>
+        <v>48616</v>
       </c>
       <c r="I15" s="23" t="n">
-        <v>25.7</v>
+        <v>16.5</v>
       </c>
       <c r="J15" s="23" t="n">
-        <v>15503</v>
+        <v>9942</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>1609</v>
+        <v>1399</v>
       </c>
       <c r="M15" s="25" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>805</v>
+        <v>333</v>
       </c>
       <c r="O15" s="26" t="n">
-        <v>29.7</v>
+        <v>19.4</v>
       </c>
       <c r="P15" s="26" t="n">
-        <v>17917</v>
+        <v>11673</v>
       </c>
       <c r="Q15" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -1733,22 +1733,22 @@
         <v>117626</v>
       </c>
       <c r="G16" s="22" t="n">
-        <v>93.2</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>109676</v>
+        <v>110508</v>
       </c>
       <c r="I16" s="23" t="n">
-        <v>6.8</v>
+        <v>5.4</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>7950</v>
+        <v>6339</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>0</v>
+        <v>779</v>
       </c>
       <c r="M16" s="25" t="n">
         <v>0</v>
@@ -1757,10 +1757,10 @@
         <v>0</v>
       </c>
       <c r="O16" s="26" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="P16" s="26" t="n">
-        <v>7950</v>
+        <v>7118</v>
       </c>
       <c r="Q16" s="27" t="inlineStr">
         <is>
@@ -1782,34 +1782,34 @@
         <v>83999</v>
       </c>
       <c r="G17" s="22" t="n">
-        <v>74.3</v>
+        <v>78.7</v>
       </c>
       <c r="H17" s="22" t="n">
-        <v>62379</v>
+        <v>66075</v>
       </c>
       <c r="I17" s="23" t="n">
-        <v>24.8</v>
+        <v>20.8</v>
       </c>
       <c r="J17" s="23" t="n">
-        <v>20865</v>
+        <v>17494</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>377</v>
+        <v>215</v>
       </c>
       <c r="M17" s="25" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="N17" s="25" t="n">
-        <v>377</v>
+        <v>215</v>
       </c>
       <c r="O17" s="26" t="n">
-        <v>25.7</v>
+        <v>21.3</v>
       </c>
       <c r="P17" s="26" t="n">
-        <v>21620</v>
+        <v>17924</v>
       </c>
       <c r="Q17" s="27" t="inlineStr">
         <is>
@@ -1831,34 +1831,34 @@
         <v>21943</v>
       </c>
       <c r="G18" s="22" t="n">
-        <v>54</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>11860</v>
+        <v>16477</v>
       </c>
       <c r="I18" s="23" t="n">
-        <v>43.6</v>
+        <v>16.7</v>
       </c>
       <c r="J18" s="23" t="n">
-        <v>9573</v>
+        <v>3664</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.2</v>
+        <v>4.8</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>44</v>
+        <v>1048</v>
       </c>
       <c r="M18" s="25" t="n">
-        <v>2.1</v>
+        <v>3.4</v>
       </c>
       <c r="N18" s="25" t="n">
-        <v>466</v>
+        <v>754</v>
       </c>
       <c r="O18" s="26" t="n">
-        <v>46</v>
+        <v>24.9</v>
       </c>
       <c r="P18" s="26" t="n">
-        <v>10083</v>
+        <v>5466</v>
       </c>
       <c r="Q18" s="27" t="inlineStr">
         <is>
@@ -1880,16 +1880,16 @@
         <v>96066</v>
       </c>
       <c r="G19" s="22" t="n">
-        <v>71.2</v>
+        <v>68.7</v>
       </c>
       <c r="H19" s="22" t="n">
-        <v>68374</v>
+        <v>65992</v>
       </c>
       <c r="I19" s="23" t="n">
-        <v>28.8</v>
+        <v>31.3</v>
       </c>
       <c r="J19" s="23" t="n">
-        <v>27692</v>
+        <v>30074</v>
       </c>
       <c r="K19" s="24" t="n">
         <v>0</v>
@@ -1904,10 +1904,10 @@
         <v>0</v>
       </c>
       <c r="O19" s="26" t="n">
-        <v>28.8</v>
+        <v>31.3</v>
       </c>
       <c r="P19" s="26" t="n">
-        <v>27692</v>
+        <v>30074</v>
       </c>
       <c r="Q19" s="27" t="inlineStr">
         <is>
@@ -1929,38 +1929,38 @@
         <v>36735</v>
       </c>
       <c r="G20" s="22" t="n">
-        <v>73.5</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="H20" s="22" t="n">
-        <v>27011</v>
+        <v>30093</v>
       </c>
       <c r="I20" s="23" t="n">
-        <v>22.8</v>
+        <v>13.9</v>
       </c>
       <c r="J20" s="23" t="n">
-        <v>8379</v>
+        <v>5113</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>1155</v>
+        <v>1412</v>
       </c>
       <c r="M20" s="25" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="N20" s="25" t="n">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="O20" s="26" t="n">
-        <v>26.5</v>
+        <v>18.1</v>
       </c>
       <c r="P20" s="26" t="n">
-        <v>9724</v>
+        <v>6642</v>
       </c>
       <c r="Q20" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -1978,22 +1978,22 @@
         <v>47297</v>
       </c>
       <c r="G21" s="22" t="n">
-        <v>93.90000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="H21" s="22" t="n">
-        <v>44426</v>
+        <v>43734</v>
       </c>
       <c r="I21" s="23" t="n">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="J21" s="23" t="n">
-        <v>2871</v>
+        <v>3461</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="M21" s="25" t="n">
         <v>0</v>
@@ -2002,10 +2002,10 @@
         <v>0</v>
       </c>
       <c r="O21" s="26" t="n">
-        <v>6.1</v>
+        <v>7.5</v>
       </c>
       <c r="P21" s="26" t="n">
-        <v>2871</v>
+        <v>3563</v>
       </c>
       <c r="Q21" s="27" t="inlineStr">
         <is>
@@ -2027,22 +2027,22 @@
         <v>53134</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>83.40000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="H22" s="22" t="n">
-        <v>44332</v>
+        <v>44883</v>
       </c>
       <c r="I22" s="23" t="n">
-        <v>16.6</v>
+        <v>14.6</v>
       </c>
       <c r="J22" s="23" t="n">
-        <v>8802</v>
+        <v>7769</v>
       </c>
       <c r="K22" s="24" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="M22" s="25" t="n">
         <v>0</v>
@@ -2051,10 +2051,10 @@
         <v>0</v>
       </c>
       <c r="O22" s="26" t="n">
-        <v>16.6</v>
+        <v>15.5</v>
       </c>
       <c r="P22" s="26" t="n">
-        <v>8802</v>
+        <v>8251</v>
       </c>
       <c r="Q22" s="27" t="inlineStr">
         <is>
@@ -2076,38 +2076,38 @@
         <v>21445</v>
       </c>
       <c r="G23" s="22" t="n">
-        <v>72.40000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="H23" s="22" t="n">
-        <v>15521</v>
+        <v>18758</v>
       </c>
       <c r="I23" s="23" t="n">
-        <v>26.8</v>
+        <v>12.4</v>
       </c>
       <c r="J23" s="23" t="n">
-        <v>5741</v>
+        <v>2664</v>
       </c>
       <c r="K23" s="24" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="M23" s="25" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>183</v>
+        <v>3</v>
       </c>
       <c r="O23" s="26" t="n">
-        <v>27.6</v>
+        <v>12.5</v>
       </c>
       <c r="P23" s="26" t="n">
-        <v>5924</v>
+        <v>2687</v>
       </c>
       <c r="Q23" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -2125,34 +2125,34 @@
         <v>186619</v>
       </c>
       <c r="G24" s="22" t="n">
-        <v>72.59999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="H24" s="22" t="n">
-        <v>135548</v>
+        <v>137579</v>
       </c>
       <c r="I24" s="23" t="n">
-        <v>26.4</v>
+        <v>24</v>
       </c>
       <c r="J24" s="23" t="n">
-        <v>49320</v>
+        <v>44816</v>
       </c>
       <c r="K24" s="24" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="L24" s="24" t="n">
-        <v>0</v>
+        <v>2241</v>
       </c>
       <c r="M24" s="25" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="N24" s="25" t="n">
-        <v>1751</v>
+        <v>1982</v>
       </c>
       <c r="O24" s="26" t="n">
-        <v>27.4</v>
+        <v>26.3</v>
       </c>
       <c r="P24" s="26" t="n">
-        <v>51071</v>
+        <v>49040</v>
       </c>
       <c r="Q24" s="27" t="inlineStr">
         <is>
@@ -2174,34 +2174,34 @@
         <v>152674</v>
       </c>
       <c r="G25" s="29" t="n">
-        <v>72.3</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="H25" s="29" t="n">
-        <v>110455</v>
+        <v>121527</v>
       </c>
       <c r="I25" s="30" t="n">
-        <v>26</v>
+        <v>19.5</v>
       </c>
       <c r="J25" s="30" t="n">
-        <v>39654</v>
+        <v>29809</v>
       </c>
       <c r="K25" s="31" t="n">
-        <v>1.6</v>
+        <v>0.8</v>
       </c>
       <c r="L25" s="31" t="n">
-        <v>2492</v>
+        <v>1240</v>
       </c>
       <c r="M25" s="32" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="N25" s="32" t="n">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="O25" s="33" t="n">
-        <v>27.7</v>
+        <v>20.4</v>
       </c>
       <c r="P25" s="33" t="n">
-        <v>42219</v>
+        <v>31147</v>
       </c>
       <c r="Q25" s="27" t="inlineStr">
         <is>
@@ -2347,22 +2347,22 @@
         <v>10163</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>67.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>6885</v>
+        <v>7259</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>32.3</v>
+        <v>24.2</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>3278</v>
+        <v>2462</v>
       </c>
       <c r="L6" s="24" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="M6" s="24" t="n">
-        <v>0</v>
+        <v>442</v>
       </c>
       <c r="N6" s="25" t="n">
         <v>0</v>
@@ -2371,10 +2371,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="26" t="n">
-        <v>32.3</v>
+        <v>28.6</v>
       </c>
       <c r="Q6" s="26" t="n">
-        <v>3278</v>
+        <v>2904</v>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
@@ -2401,22 +2401,22 @@
         <v>99852</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>94.3</v>
+        <v>96.2</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>94146</v>
+        <v>96075</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>5.7</v>
+        <v>3.3</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>5706</v>
+        <v>3313</v>
       </c>
       <c r="L7" s="24" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M7" s="24" t="n">
-        <v>0</v>
+        <v>464</v>
       </c>
       <c r="N7" s="25" t="n">
         <v>0</v>
@@ -2425,10 +2425,10 @@
         <v>0</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
       <c r="Q7" s="26" t="n">
-        <v>5706</v>
+        <v>3777</v>
       </c>
       <c r="R7" s="27" t="inlineStr">
         <is>
@@ -2455,16 +2455,16 @@
         <v>50005</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>82.3</v>
+        <v>85.5</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>41164</v>
+        <v>42731</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>17.7</v>
+        <v>14.5</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>8841</v>
+        <v>7274</v>
       </c>
       <c r="L8" s="24" t="n">
         <v>0</v>
@@ -2479,10 +2479,10 @@
         <v>0</v>
       </c>
       <c r="P8" s="26" t="n">
-        <v>17.7</v>
+        <v>14.5</v>
       </c>
       <c r="Q8" s="26" t="n">
-        <v>8841</v>
+        <v>7274</v>
       </c>
       <c r="R8" s="27" t="inlineStr">
         <is>
@@ -2509,16 +2509,16 @@
         <v>66985</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>85.59999999999999</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="I9" s="22" t="n">
-        <v>57341</v>
+        <v>57232</v>
       </c>
       <c r="J9" s="23" t="n">
-        <v>14</v>
+        <v>14.1</v>
       </c>
       <c r="K9" s="23" t="n">
-        <v>9383</v>
+        <v>9463</v>
       </c>
       <c r="L9" s="24" t="n">
         <v>0</v>
@@ -2530,13 +2530,13 @@
         <v>0.4</v>
       </c>
       <c r="O9" s="25" t="n">
-        <v>261</v>
+        <v>291</v>
       </c>
       <c r="P9" s="26" t="n">
-        <v>14.4</v>
+        <v>14.6</v>
       </c>
       <c r="Q9" s="26" t="n">
-        <v>9644</v>
+        <v>9753</v>
       </c>
       <c r="R9" s="27" t="inlineStr">
         <is>
@@ -2563,22 +2563,22 @@
         <v>95309</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>82.3</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>78431</v>
+        <v>81896</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>16.1</v>
+        <v>13.4</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>15388</v>
+        <v>12782</v>
       </c>
       <c r="L10" s="24" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="M10" s="24" t="n">
-        <v>1489</v>
+        <v>631</v>
       </c>
       <c r="N10" s="25" t="n">
         <v>0</v>
@@ -2587,10 +2587,10 @@
         <v>0</v>
       </c>
       <c r="P10" s="26" t="n">
-        <v>17.7</v>
+        <v>14.1</v>
       </c>
       <c r="Q10" s="26" t="n">
-        <v>16878</v>
+        <v>13413</v>
       </c>
       <c r="R10" s="27" t="inlineStr">
         <is>
@@ -2617,16 +2617,16 @@
         <v>5527</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>96.5</v>
+        <v>97.8</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>5333</v>
+        <v>5407</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>3.5</v>
+        <v>2.2</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>194</v>
+        <v>120</v>
       </c>
       <c r="L11" s="24" t="n">
         <v>0</v>
@@ -2641,10 +2641,10 @@
         <v>0</v>
       </c>
       <c r="P11" s="26" t="n">
-        <v>3.5</v>
+        <v>2.2</v>
       </c>
       <c r="Q11" s="26" t="n">
-        <v>194</v>
+        <v>120</v>
       </c>
       <c r="R11" s="27" t="inlineStr">
         <is>
@@ -2671,34 +2671,34 @@
         <v>515</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>81.7</v>
+        <v>80</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>17.8</v>
+        <v>16.5</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="M12" s="24" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="N12" s="25" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P12" s="26" t="n">
-        <v>18.3</v>
+        <v>20</v>
       </c>
       <c r="Q12" s="26" t="n">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="R12" s="27" t="inlineStr">
         <is>
@@ -2725,22 +2725,22 @@
         <v>27794</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>69.40000000000001</v>
+        <v>72.7</v>
       </c>
       <c r="I13" s="22" t="n">
-        <v>19294</v>
+        <v>20216</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>30.6</v>
+        <v>13</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>8500</v>
+        <v>3615</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>0</v>
+        <v>3963</v>
       </c>
       <c r="N13" s="25" t="n">
         <v>0</v>
@@ -2749,10 +2749,10 @@
         <v>0</v>
       </c>
       <c r="P13" s="26" t="n">
-        <v>30.6</v>
+        <v>27.3</v>
       </c>
       <c r="Q13" s="26" t="n">
-        <v>8500</v>
+        <v>7578</v>
       </c>
       <c r="R13" s="27" t="inlineStr">
         <is>
@@ -2779,16 +2779,16 @@
         <v>7901</v>
       </c>
       <c r="H14" s="22" t="n">
-        <v>59</v>
+        <v>54.4</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>4661</v>
+        <v>4302</v>
       </c>
       <c r="J14" s="23" t="n">
-        <v>41</v>
+        <v>45.6</v>
       </c>
       <c r="K14" s="23" t="n">
-        <v>3240</v>
+        <v>3599</v>
       </c>
       <c r="L14" s="24" t="n">
         <v>0</v>
@@ -2803,10 +2803,10 @@
         <v>0</v>
       </c>
       <c r="P14" s="26" t="n">
-        <v>41</v>
+        <v>45.6</v>
       </c>
       <c r="Q14" s="26" t="n">
-        <v>3240</v>
+        <v>3599</v>
       </c>
       <c r="R14" s="27" t="inlineStr">
         <is>
@@ -2833,22 +2833,22 @@
         <v>108049</v>
       </c>
       <c r="H15" s="22" t="n">
-        <v>93.5</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I15" s="22" t="n">
-        <v>101011</v>
+        <v>101961</v>
       </c>
       <c r="J15" s="23" t="n">
-        <v>6.5</v>
+        <v>5.1</v>
       </c>
       <c r="K15" s="23" t="n">
-        <v>7038</v>
+        <v>5458</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>0</v>
+        <v>630</v>
       </c>
       <c r="N15" s="25" t="n">
         <v>0</v>
@@ -2857,10 +2857,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="26" t="n">
-        <v>6.5</v>
+        <v>5.6</v>
       </c>
       <c r="Q15" s="26" t="n">
-        <v>7038</v>
+        <v>6088</v>
       </c>
       <c r="R15" s="27" t="inlineStr">
         <is>
@@ -2887,16 +2887,16 @@
         <v>45116</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>72.5</v>
+        <v>76.2</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>32693</v>
+        <v>34374</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>27.5</v>
+        <v>23.8</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>12423</v>
+        <v>10742</v>
       </c>
       <c r="L16" s="24" t="n">
         <v>0</v>
@@ -2911,10 +2911,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="26" t="n">
-        <v>27.5</v>
+        <v>23.8</v>
       </c>
       <c r="Q16" s="26" t="n">
-        <v>12423</v>
+        <v>10742</v>
       </c>
       <c r="R16" s="27" t="inlineStr">
         <is>
@@ -2941,16 +2941,16 @@
         <v>2358</v>
       </c>
       <c r="H17" s="22" t="n">
-        <v>76.90000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="I17" s="22" t="n">
-        <v>1814</v>
+        <v>1918</v>
       </c>
       <c r="J17" s="23" t="n">
-        <v>23.1</v>
+        <v>18.6</v>
       </c>
       <c r="K17" s="23" t="n">
-        <v>544</v>
+        <v>440</v>
       </c>
       <c r="L17" s="24" t="n">
         <v>0</v>
@@ -2965,14 +2965,14 @@
         <v>0</v>
       </c>
       <c r="P17" s="26" t="n">
-        <v>23.1</v>
+        <v>18.6</v>
       </c>
       <c r="Q17" s="26" t="n">
-        <v>544</v>
+        <v>440</v>
       </c>
       <c r="R17" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -2995,16 +2995,16 @@
         <v>95228</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>71</v>
+        <v>68.5</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>67648</v>
+        <v>65261</v>
       </c>
       <c r="J18" s="23" t="n">
-        <v>29</v>
+        <v>31.5</v>
       </c>
       <c r="K18" s="23" t="n">
-        <v>27580</v>
+        <v>29967</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>0</v>
@@ -3019,10 +3019,10 @@
         <v>0</v>
       </c>
       <c r="P18" s="26" t="n">
-        <v>29</v>
+        <v>31.5</v>
       </c>
       <c r="Q18" s="26" t="n">
-        <v>27580</v>
+        <v>29967</v>
       </c>
       <c r="R18" s="27" t="inlineStr">
         <is>
@@ -3049,22 +3049,22 @@
         <v>13103</v>
       </c>
       <c r="H19" s="22" t="n">
-        <v>66.09999999999999</v>
+        <v>80.5</v>
       </c>
       <c r="I19" s="22" t="n">
-        <v>8660</v>
+        <v>10553</v>
       </c>
       <c r="J19" s="23" t="n">
-        <v>31.6</v>
+        <v>18</v>
       </c>
       <c r="K19" s="23" t="n">
-        <v>4142</v>
+        <v>2354</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>2.3</v>
+        <v>1.5</v>
       </c>
       <c r="M19" s="24" t="n">
-        <v>301</v>
+        <v>196</v>
       </c>
       <c r="N19" s="25" t="n">
         <v>0</v>
@@ -3073,14 +3073,14 @@
         <v>0</v>
       </c>
       <c r="P19" s="26" t="n">
-        <v>33.9</v>
+        <v>19.5</v>
       </c>
       <c r="Q19" s="26" t="n">
-        <v>4443</v>
+        <v>2550</v>
       </c>
       <c r="R19" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -3103,22 +3103,22 @@
         <v>10079</v>
       </c>
       <c r="H20" s="22" t="n">
-        <v>91.8</v>
+        <v>93.2</v>
       </c>
       <c r="I20" s="22" t="n">
-        <v>9250</v>
+        <v>9390</v>
       </c>
       <c r="J20" s="23" t="n">
-        <v>8.199999999999999</v>
+        <v>5.8</v>
       </c>
       <c r="K20" s="23" t="n">
-        <v>829</v>
+        <v>587</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="24" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="N20" s="25" t="n">
         <v>0</v>
@@ -3127,10 +3127,10 @@
         <v>0</v>
       </c>
       <c r="P20" s="26" t="n">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="Q20" s="26" t="n">
-        <v>829</v>
+        <v>689</v>
       </c>
       <c r="R20" s="27" t="inlineStr">
         <is>
@@ -3157,22 +3157,22 @@
         <v>32621</v>
       </c>
       <c r="H21" s="22" t="n">
-        <v>83.09999999999999</v>
+        <v>86</v>
       </c>
       <c r="I21" s="22" t="n">
-        <v>27122</v>
+        <v>28055</v>
       </c>
       <c r="J21" s="23" t="n">
-        <v>16.9</v>
+        <v>13.1</v>
       </c>
       <c r="K21" s="23" t="n">
-        <v>5499</v>
+        <v>4262</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="M21" s="24" t="n">
-        <v>0</v>
+        <v>304</v>
       </c>
       <c r="N21" s="25" t="n">
         <v>0</v>
@@ -3181,10 +3181,10 @@
         <v>0</v>
       </c>
       <c r="P21" s="26" t="n">
-        <v>16.9</v>
+        <v>14</v>
       </c>
       <c r="Q21" s="26" t="n">
-        <v>5499</v>
+        <v>4566</v>
       </c>
       <c r="R21" s="27" t="inlineStr">
         <is>
@@ -3211,38 +3211,38 @@
         <v>1240</v>
       </c>
       <c r="H22" s="22" t="n">
-        <v>67.09999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>832</v>
+        <v>993</v>
       </c>
       <c r="J22" s="23" t="n">
-        <v>32.2</v>
+        <v>18.9</v>
       </c>
       <c r="K22" s="23" t="n">
-        <v>399</v>
+        <v>235</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N22" s="25" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="O22" s="25" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="P22" s="26" t="n">
-        <v>32.9</v>
+        <v>19.9</v>
       </c>
       <c r="Q22" s="26" t="n">
-        <v>408</v>
+        <v>247</v>
       </c>
       <c r="R22" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -3265,34 +3265,34 @@
         <v>177704</v>
       </c>
       <c r="H23" s="22" t="n">
-        <v>72.90000000000001</v>
+        <v>74</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>129558</v>
+        <v>131543</v>
       </c>
       <c r="J23" s="23" t="n">
-        <v>26.1</v>
+        <v>23.7</v>
       </c>
       <c r="K23" s="23" t="n">
-        <v>46396</v>
+        <v>42054</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="M23" s="24" t="n">
-        <v>0</v>
+        <v>2124</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>1751</v>
+        <v>1982</v>
       </c>
       <c r="P23" s="26" t="n">
-        <v>27.1</v>
+        <v>26</v>
       </c>
       <c r="Q23" s="26" t="n">
-        <v>48146</v>
+        <v>46161</v>
       </c>
       <c r="R23" s="27" t="inlineStr">
         <is>
@@ -3319,22 +3319,22 @@
         <v>142058</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>72.8</v>
+        <v>79.8</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>103428</v>
+        <v>113294</v>
       </c>
       <c r="J24" s="30" t="n">
-        <v>25.4</v>
+        <v>19.4</v>
       </c>
       <c r="K24" s="30" t="n">
-        <v>36138</v>
+        <v>27590</v>
       </c>
       <c r="L24" s="31" t="n">
-        <v>1.8</v>
+        <v>0.8</v>
       </c>
       <c r="M24" s="31" t="n">
-        <v>2492</v>
+        <v>1174</v>
       </c>
       <c r="N24" s="32" t="n">
         <v>0</v>
@@ -3343,10 +3343,10 @@
         <v>0</v>
       </c>
       <c r="P24" s="33" t="n">
-        <v>27.2</v>
+        <v>20.2</v>
       </c>
       <c r="Q24" s="33" t="n">
-        <v>38630</v>
+        <v>28764</v>
       </c>
       <c r="R24" s="27" t="inlineStr">
         <is>
@@ -3492,22 +3492,22 @@
         <v>10127</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>92.59999999999999</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>9381</v>
+        <v>9918</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>7.4</v>
+        <v>1.9</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>746</v>
+        <v>189</v>
       </c>
       <c r="L6" s="24" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="M6" s="24" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N6" s="25" t="n">
         <v>0</v>
@@ -3516,10 +3516,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="26" t="n">
-        <v>7.4</v>
+        <v>2.1</v>
       </c>
       <c r="Q6" s="26" t="n">
-        <v>746</v>
+        <v>209</v>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
@@ -3546,38 +3546,38 @@
         <v>13449</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>55.9</v>
+        <v>56.7</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>7521</v>
+        <v>7619</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>23</v>
+        <v>23.7</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>3097</v>
+        <v>3186</v>
       </c>
       <c r="L7" s="24" t="n">
         <v>0.7</v>
       </c>
       <c r="M7" s="24" t="n">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>20.4</v>
+        <v>18.9</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>2743</v>
+        <v>2545</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>44.1</v>
+        <v>43.3</v>
       </c>
       <c r="Q7" s="26" t="n">
-        <v>5928</v>
+        <v>5830</v>
       </c>
       <c r="R7" s="27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -3600,16 +3600,16 @@
         <v>2823</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>88.59999999999999</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>2502</v>
+        <v>2497</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="L8" s="24" t="n">
         <v>0</v>
@@ -3624,10 +3624,10 @@
         <v>0</v>
       </c>
       <c r="P8" s="26" t="n">
-        <v>11.4</v>
+        <v>11.6</v>
       </c>
       <c r="Q8" s="26" t="n">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="R8" s="27" t="inlineStr">
         <is>
@@ -3654,22 +3654,22 @@
         <v>7936</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>75.40000000000001</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="I9" s="22" t="n">
-        <v>5985</v>
+        <v>6938</v>
       </c>
       <c r="J9" s="23" t="n">
-        <v>23.5</v>
+        <v>12.6</v>
       </c>
       <c r="K9" s="23" t="n">
-        <v>1865</v>
+        <v>998</v>
       </c>
       <c r="L9" s="24" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="M9" s="24" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="N9" s="25" t="n">
         <v>0</v>
@@ -3678,14 +3678,14 @@
         <v>0</v>
       </c>
       <c r="P9" s="26" t="n">
-        <v>24.6</v>
+        <v>12.6</v>
       </c>
       <c r="Q9" s="26" t="n">
-        <v>1951</v>
+        <v>998</v>
       </c>
       <c r="R9" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -3708,16 +3708,16 @@
         <v>5818</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>97.09999999999999</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>5651</v>
+        <v>5680</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>2.3</v>
+        <v>1.6</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>134</v>
+        <v>96</v>
       </c>
       <c r="L10" s="24" t="n">
         <v>0</v>
@@ -3726,16 +3726,16 @@
         <v>0</v>
       </c>
       <c r="N10" s="25" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="O10" s="25" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="P10" s="26" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="Q10" s="26" t="n">
-        <v>167</v>
+        <v>138</v>
       </c>
       <c r="R10" s="27" t="inlineStr">
         <is>
@@ -3762,34 +3762,34 @@
         <v>32072</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>59.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>19150</v>
+        <v>22644</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>39.3</v>
+        <v>25.3</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>12611</v>
+        <v>8115</v>
       </c>
       <c r="L11" s="24" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="M11" s="24" t="n">
-        <v>0</v>
+        <v>1005</v>
       </c>
       <c r="N11" s="25" t="n">
         <v>1</v>
       </c>
       <c r="O11" s="25" t="n">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="P11" s="26" t="n">
-        <v>40.3</v>
+        <v>29.4</v>
       </c>
       <c r="Q11" s="26" t="n">
-        <v>12922</v>
+        <v>9428</v>
       </c>
       <c r="R11" s="27" t="inlineStr">
         <is>
@@ -3816,22 +3816,22 @@
         <v>4224</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>65.09999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>2751</v>
+        <v>2888</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>34.9</v>
+        <v>7.4</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>1473</v>
+        <v>310</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>0</v>
+        <v>24.3</v>
       </c>
       <c r="M12" s="24" t="n">
-        <v>0</v>
+        <v>1025</v>
       </c>
       <c r="N12" s="25" t="n">
         <v>0</v>
@@ -3840,14 +3840,14 @@
         <v>0</v>
       </c>
       <c r="P12" s="26" t="n">
-        <v>34.9</v>
+        <v>31.6</v>
       </c>
       <c r="Q12" s="26" t="n">
-        <v>1473</v>
+        <v>1336</v>
       </c>
       <c r="R12" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -3870,34 +3870,34 @@
         <v>3204</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>55.6</v>
+        <v>60.6</v>
       </c>
       <c r="I13" s="22" t="n">
-        <v>1780</v>
+        <v>1942</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>43.3</v>
+        <v>38.7</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>1388</v>
+        <v>1240</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="N13" s="25" t="n">
-        <v>1.1</v>
+        <v>0.5</v>
       </c>
       <c r="O13" s="25" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="P13" s="26" t="n">
-        <v>44.4</v>
+        <v>39.4</v>
       </c>
       <c r="Q13" s="26" t="n">
-        <v>1424</v>
+        <v>1262</v>
       </c>
       <c r="R13" s="27" t="inlineStr">
         <is>
@@ -3978,22 +3978,22 @@
         <v>9577</v>
       </c>
       <c r="H15" s="22" t="n">
-        <v>90.5</v>
+        <v>89.2</v>
       </c>
       <c r="I15" s="22" t="n">
-        <v>8665</v>
+        <v>8547</v>
       </c>
       <c r="J15" s="23" t="n">
-        <v>9.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K15" s="23" t="n">
-        <v>912</v>
+        <v>881</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="N15" s="25" t="n">
         <v>0</v>
@@ -4002,10 +4002,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="26" t="n">
-        <v>9.5</v>
+        <v>10.8</v>
       </c>
       <c r="Q15" s="26" t="n">
-        <v>912</v>
+        <v>1030</v>
       </c>
       <c r="R15" s="27" t="inlineStr">
         <is>
@@ -4032,16 +4032,16 @@
         <v>18886</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>65.3</v>
+        <v>76.2</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>12331</v>
+        <v>14392</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>34.7</v>
+        <v>23.8</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>6555</v>
+        <v>4494</v>
       </c>
       <c r="L16" s="24" t="n">
         <v>0</v>
@@ -4056,10 +4056,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="26" t="n">
-        <v>34.7</v>
+        <v>23.8</v>
       </c>
       <c r="Q16" s="26" t="n">
-        <v>6555</v>
+        <v>4494</v>
       </c>
       <c r="R16" s="27" t="inlineStr">
         <is>
@@ -4086,34 +4086,34 @@
         <v>4256</v>
       </c>
       <c r="H17" s="22" t="n">
-        <v>69.3</v>
+        <v>79.8</v>
       </c>
       <c r="I17" s="22" t="n">
-        <v>2948</v>
+        <v>3395</v>
       </c>
       <c r="J17" s="23" t="n">
-        <v>29.2</v>
+        <v>15.7</v>
       </c>
       <c r="K17" s="23" t="n">
-        <v>1241</v>
+        <v>669</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>1</v>
+        <v>3.7</v>
       </c>
       <c r="M17" s="24" t="n">
-        <v>44</v>
+        <v>159</v>
       </c>
       <c r="N17" s="25" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="O17" s="25" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="P17" s="26" t="n">
-        <v>30.7</v>
+        <v>20.2</v>
       </c>
       <c r="Q17" s="26" t="n">
-        <v>1308</v>
+        <v>861</v>
       </c>
       <c r="R17" s="27" t="inlineStr">
         <is>
@@ -4140,16 +4140,16 @@
         <v>838</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>86.59999999999999</v>
+        <v>87.3</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="J18" s="23" t="n">
-        <v>13.4</v>
+        <v>12.7</v>
       </c>
       <c r="K18" s="23" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>0</v>
@@ -4164,10 +4164,10 @@
         <v>0</v>
       </c>
       <c r="P18" s="26" t="n">
-        <v>13.4</v>
+        <v>12.7</v>
       </c>
       <c r="Q18" s="26" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="R18" s="27" t="inlineStr">
         <is>
@@ -4194,38 +4194,38 @@
         <v>18466</v>
       </c>
       <c r="H19" s="22" t="n">
-        <v>75.3</v>
+        <v>80.7</v>
       </c>
       <c r="I19" s="22" t="n">
-        <v>13908</v>
+        <v>14906</v>
       </c>
       <c r="J19" s="23" t="n">
-        <v>19.6</v>
+        <v>13.4</v>
       </c>
       <c r="K19" s="23" t="n">
-        <v>3623</v>
+        <v>2474</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>4.4</v>
+        <v>5.6</v>
       </c>
       <c r="M19" s="24" t="n">
-        <v>818</v>
+        <v>1026</v>
       </c>
       <c r="N19" s="25" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="O19" s="25" t="n">
-        <v>117</v>
+        <v>60</v>
       </c>
       <c r="P19" s="26" t="n">
-        <v>24.7</v>
+        <v>19.3</v>
       </c>
       <c r="Q19" s="26" t="n">
-        <v>4558</v>
+        <v>3560</v>
       </c>
       <c r="R19" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -4302,22 +4302,22 @@
         <v>20513</v>
       </c>
       <c r="H21" s="22" t="n">
-        <v>83.90000000000001</v>
+        <v>82</v>
       </c>
       <c r="I21" s="22" t="n">
-        <v>17210</v>
+        <v>16828</v>
       </c>
       <c r="J21" s="23" t="n">
-        <v>16.1</v>
+        <v>17.1</v>
       </c>
       <c r="K21" s="23" t="n">
-        <v>3303</v>
+        <v>3508</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="M21" s="24" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="N21" s="25" t="n">
         <v>0</v>
@@ -4326,10 +4326,10 @@
         <v>0</v>
       </c>
       <c r="P21" s="26" t="n">
-        <v>16.1</v>
+        <v>18</v>
       </c>
       <c r="Q21" s="26" t="n">
-        <v>3303</v>
+        <v>3685</v>
       </c>
       <c r="R21" s="27" t="inlineStr">
         <is>
@@ -4356,22 +4356,22 @@
         <v>784</v>
       </c>
       <c r="H22" s="22" t="n">
-        <v>74</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="I22" s="22" t="n">
-        <v>580</v>
+        <v>613</v>
       </c>
       <c r="J22" s="23" t="n">
-        <v>26</v>
+        <v>20.5</v>
       </c>
       <c r="K22" s="23" t="n">
-        <v>204</v>
+        <v>161</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N22" s="25" t="n">
         <v>0</v>
@@ -4380,10 +4380,10 @@
         <v>0</v>
       </c>
       <c r="P22" s="26" t="n">
-        <v>26</v>
+        <v>21.9</v>
       </c>
       <c r="Q22" s="26" t="n">
-        <v>204</v>
+        <v>171</v>
       </c>
       <c r="R22" s="27" t="inlineStr">
         <is>
@@ -4410,16 +4410,16 @@
         <v>1952</v>
       </c>
       <c r="H23" s="22" t="n">
-        <v>67.40000000000001</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="I23" s="22" t="n">
-        <v>1315</v>
+        <v>1285</v>
       </c>
       <c r="J23" s="23" t="n">
-        <v>32.6</v>
+        <v>34.1</v>
       </c>
       <c r="K23" s="23" t="n">
-        <v>637</v>
+        <v>667</v>
       </c>
       <c r="L23" s="24" t="n">
         <v>0</v>
@@ -4434,10 +4434,10 @@
         <v>0</v>
       </c>
       <c r="P23" s="26" t="n">
-        <v>32.6</v>
+        <v>34.1</v>
       </c>
       <c r="Q23" s="26" t="n">
-        <v>637</v>
+        <v>667</v>
       </c>
       <c r="R23" s="27" t="inlineStr">
         <is>
@@ -4464,16 +4464,16 @@
         <v>1284</v>
       </c>
       <c r="H24" s="29" t="n">
-        <v>85.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="I24" s="29" t="n">
-        <v>1095</v>
+        <v>1161</v>
       </c>
       <c r="J24" s="30" t="n">
-        <v>14.7</v>
+        <v>9.6</v>
       </c>
       <c r="K24" s="30" t="n">
-        <v>189</v>
+        <v>123</v>
       </c>
       <c r="L24" s="31" t="n">
         <v>0</v>
@@ -4488,10 +4488,10 @@
         <v>0</v>
       </c>
       <c r="P24" s="33" t="n">
-        <v>14.7</v>
+        <v>9.6</v>
       </c>
       <c r="Q24" s="33" t="n">
-        <v>189</v>
+        <v>123</v>
       </c>
       <c r="R24" s="27" t="inlineStr">
         <is>
@@ -4637,22 +4637,22 @@
         <v>1311</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>56.8</v>
+        <v>63.2</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>745</v>
+        <v>828</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>42.1</v>
+        <v>26.9</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>552</v>
+        <v>352</v>
       </c>
       <c r="L6" s="24" t="n">
-        <v>1.1</v>
+        <v>9.9</v>
       </c>
       <c r="M6" s="24" t="n">
-        <v>14</v>
+        <v>130</v>
       </c>
       <c r="N6" s="25" t="n">
         <v>0</v>
@@ -4661,10 +4661,10 @@
         <v>0</v>
       </c>
       <c r="P6" s="26" t="n">
-        <v>43.2</v>
+        <v>36.8</v>
       </c>
       <c r="Q6" s="26" t="n">
-        <v>566</v>
+        <v>483</v>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
@@ -4691,16 +4691,16 @@
         <v>11032</v>
       </c>
       <c r="H7" s="22" t="n">
-        <v>93</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="I7" s="22" t="n">
-        <v>10256</v>
+        <v>10440</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
       <c r="K7" s="23" t="n">
-        <v>603</v>
+        <v>592</v>
       </c>
       <c r="L7" s="24" t="n">
         <v>0</v>
@@ -4709,16 +4709,16 @@
         <v>0</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="P7" s="26" t="n">
-        <v>7</v>
+        <v>5.4</v>
       </c>
       <c r="Q7" s="26" t="n">
-        <v>776</v>
+        <v>592</v>
       </c>
       <c r="R7" s="27" t="inlineStr">
         <is>
@@ -4745,22 +4745,22 @@
         <v>1662</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>77.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>1284</v>
+        <v>1314</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>22.7</v>
+        <v>19.5</v>
       </c>
       <c r="K8" s="23" t="n">
-        <v>378</v>
+        <v>324</v>
       </c>
       <c r="L8" s="24" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="M8" s="24" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="N8" s="25" t="n">
         <v>0</v>
@@ -4769,10 +4769,10 @@
         <v>0</v>
       </c>
       <c r="P8" s="26" t="n">
-        <v>22.7</v>
+        <v>20.9</v>
       </c>
       <c r="Q8" s="26" t="n">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="R8" s="27" t="inlineStr">
         <is>
@@ -4799,16 +4799,16 @@
         <v>19666</v>
       </c>
       <c r="H9" s="22" t="n">
-        <v>74.8</v>
+        <v>83.7</v>
       </c>
       <c r="I9" s="22" t="n">
-        <v>14707</v>
+        <v>16455</v>
       </c>
       <c r="J9" s="23" t="n">
-        <v>25.2</v>
+        <v>16.3</v>
       </c>
       <c r="K9" s="23" t="n">
-        <v>4959</v>
+        <v>3211</v>
       </c>
       <c r="L9" s="24" t="n">
         <v>0</v>
@@ -4823,14 +4823,14 @@
         <v>0</v>
       </c>
       <c r="P9" s="26" t="n">
-        <v>25.2</v>
+        <v>16.3</v>
       </c>
       <c r="Q9" s="26" t="n">
-        <v>4959</v>
+        <v>3211</v>
       </c>
       <c r="R9" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -4853,38 +4853,38 @@
         <v>30911</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>76.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="I10" s="22" t="n">
-        <v>23655</v>
+        <v>24913</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>22.1</v>
+        <v>15</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>6821</v>
+        <v>4647</v>
       </c>
       <c r="L10" s="24" t="n">
-        <v>0.9</v>
+        <v>4</v>
       </c>
       <c r="M10" s="24" t="n">
-        <v>290</v>
+        <v>1243</v>
       </c>
       <c r="N10" s="25" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="O10" s="25" t="n">
-        <v>145</v>
+        <v>108</v>
       </c>
       <c r="P10" s="26" t="n">
-        <v>23.5</v>
+        <v>19.4</v>
       </c>
       <c r="Q10" s="26" t="n">
-        <v>7256</v>
+        <v>5998</v>
       </c>
       <c r="R10" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -4907,16 +4907,16 @@
         <v>5832</v>
       </c>
       <c r="H11" s="22" t="n">
-        <v>52.4</v>
+        <v>50.5</v>
       </c>
       <c r="I11" s="22" t="n">
-        <v>3056</v>
+        <v>2948</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>47.6</v>
+        <v>49.5</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>2776</v>
+        <v>2884</v>
       </c>
       <c r="L11" s="24" t="n">
         <v>0</v>
@@ -4931,10 +4931,10 @@
         <v>0</v>
       </c>
       <c r="P11" s="26" t="n">
-        <v>47.6</v>
+        <v>49.5</v>
       </c>
       <c r="Q11" s="26" t="n">
-        <v>2776</v>
+        <v>2884</v>
       </c>
       <c r="R11" s="27" t="inlineStr">
         <is>
@@ -4961,38 +4961,38 @@
         <v>59804</v>
       </c>
       <c r="H12" s="22" t="n">
-        <v>70.90000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="I12" s="22" t="n">
-        <v>42372</v>
+        <v>48616</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>25.1</v>
+        <v>15.8</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>15018</v>
+        <v>9457</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>2.7</v>
+        <v>2.3</v>
       </c>
       <c r="M12" s="24" t="n">
-        <v>1609</v>
+        <v>1399</v>
       </c>
       <c r="N12" s="25" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>805</v>
+        <v>333</v>
       </c>
       <c r="P12" s="26" t="n">
-        <v>29.1</v>
+        <v>18.7</v>
       </c>
       <c r="Q12" s="26" t="n">
-        <v>17432</v>
+        <v>11188</v>
       </c>
       <c r="R12" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -5015,34 +5015,34 @@
         <v>19997</v>
       </c>
       <c r="H13" s="22" t="n">
-        <v>86.8</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="I13" s="22" t="n">
-        <v>17356</v>
+        <v>17309</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>9.4</v>
+        <v>11.3</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>1887</v>
+        <v>2258</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>377</v>
+        <v>215</v>
       </c>
       <c r="N13" s="25" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="O13" s="25" t="n">
-        <v>377</v>
+        <v>215</v>
       </c>
       <c r="P13" s="26" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="Q13" s="26" t="n">
-        <v>2641</v>
+        <v>2688</v>
       </c>
       <c r="R13" s="27" t="inlineStr">
         <is>
@@ -5069,34 +5069,34 @@
         <v>15329</v>
       </c>
       <c r="H14" s="22" t="n">
-        <v>46.3</v>
+        <v>72.8</v>
       </c>
       <c r="I14" s="22" t="n">
-        <v>7098</v>
+        <v>11164</v>
       </c>
       <c r="J14" s="23" t="n">
-        <v>50.8</v>
+        <v>16.7</v>
       </c>
       <c r="K14" s="23" t="n">
-        <v>7788</v>
+        <v>2555</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="M14" s="24" t="n">
-        <v>0</v>
+        <v>889</v>
       </c>
       <c r="N14" s="25" t="n">
-        <v>2.9</v>
+        <v>4.7</v>
       </c>
       <c r="O14" s="25" t="n">
-        <v>444</v>
+        <v>722</v>
       </c>
       <c r="P14" s="26" t="n">
-        <v>53.7</v>
+        <v>27.2</v>
       </c>
       <c r="Q14" s="26" t="n">
-        <v>8231</v>
+        <v>4165</v>
       </c>
       <c r="R14" s="27" t="inlineStr">
         <is>
@@ -5123,34 +5123,34 @@
         <v>5166</v>
       </c>
       <c r="H15" s="22" t="n">
-        <v>86</v>
+        <v>89.7</v>
       </c>
       <c r="I15" s="22" t="n">
-        <v>4443</v>
+        <v>4634</v>
       </c>
       <c r="J15" s="23" t="n">
-        <v>11.9</v>
+        <v>5.5</v>
       </c>
       <c r="K15" s="23" t="n">
-        <v>614</v>
+        <v>285</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.7</v>
+        <v>3.7</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>36</v>
+        <v>190</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="O15" s="25" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="P15" s="26" t="n">
-        <v>14</v>
+        <v>10.3</v>
       </c>
       <c r="Q15" s="26" t="n">
-        <v>723</v>
+        <v>532</v>
       </c>
       <c r="R15" s="27" t="inlineStr">
         <is>
@@ -5177,16 +5177,16 @@
         <v>37056</v>
       </c>
       <c r="H16" s="22" t="n">
-        <v>94.5</v>
+        <v>92.2</v>
       </c>
       <c r="I16" s="22" t="n">
-        <v>35015</v>
+        <v>34182</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>5.5</v>
+        <v>7.8</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>2041</v>
+        <v>2874</v>
       </c>
       <c r="L16" s="24" t="n">
         <v>0</v>
@@ -5201,10 +5201,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="26" t="n">
-        <v>5.5</v>
+        <v>7.8</v>
       </c>
       <c r="Q16" s="26" t="n">
-        <v>2041</v>
+        <v>2874</v>
       </c>
       <c r="R16" s="27" t="inlineStr">
         <is>
@@ -5231,16 +5231,16 @@
         <v>19421</v>
       </c>
       <c r="H17" s="22" t="n">
-        <v>72.59999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="I17" s="22" t="n">
-        <v>14109</v>
+        <v>17152</v>
       </c>
       <c r="J17" s="23" t="n">
-        <v>26.5</v>
+        <v>11.7</v>
       </c>
       <c r="K17" s="23" t="n">
-        <v>5138</v>
+        <v>2269</v>
       </c>
       <c r="L17" s="24" t="n">
         <v>0</v>
@@ -5249,20 +5249,20 @@
         <v>0</v>
       </c>
       <c r="N17" s="25" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="O17" s="25" t="n">
-        <v>174</v>
+        <v>0</v>
       </c>
       <c r="P17" s="26" t="n">
-        <v>27.4</v>
+        <v>11.7</v>
       </c>
       <c r="Q17" s="26" t="n">
-        <v>5312</v>
+        <v>2269</v>
       </c>
       <c r="R17" s="27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -5285,22 +5285,22 @@
         <v>6963</v>
       </c>
       <c r="H18" s="22" t="n">
-        <v>67.09999999999999</v>
+        <v>68.2</v>
       </c>
       <c r="I18" s="22" t="n">
-        <v>4676</v>
+        <v>4751</v>
       </c>
       <c r="J18" s="23" t="n">
-        <v>32.9</v>
+        <v>30.1</v>
       </c>
       <c r="K18" s="23" t="n">
-        <v>2287</v>
+        <v>2096</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="M18" s="24" t="n">
-        <v>0</v>
+        <v>117</v>
       </c>
       <c r="N18" s="25" t="n">
         <v>0</v>
@@ -5309,10 +5309,10 @@
         <v>0</v>
       </c>
       <c r="P18" s="26" t="n">
-        <v>32.9</v>
+        <v>31.8</v>
       </c>
       <c r="Q18" s="26" t="n">
-        <v>2287</v>
+        <v>2212</v>
       </c>
       <c r="R18" s="27" t="inlineStr">
         <is>
@@ -5339,34 +5339,34 @@
         <v>9332</v>
       </c>
       <c r="H19" s="29" t="n">
-        <v>63.6</v>
+        <v>75.8</v>
       </c>
       <c r="I19" s="29" t="n">
-        <v>5932</v>
+        <v>7073</v>
       </c>
       <c r="J19" s="30" t="n">
-        <v>35.7</v>
+        <v>22.5</v>
       </c>
       <c r="K19" s="30" t="n">
-        <v>3328</v>
+        <v>2096</v>
       </c>
       <c r="L19" s="31" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="M19" s="31" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="N19" s="32" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
       <c r="O19" s="32" t="n">
-        <v>72</v>
+        <v>98</v>
       </c>
       <c r="P19" s="33" t="n">
-        <v>36.4</v>
+        <v>24.2</v>
       </c>
       <c r="Q19" s="33" t="n">
-        <v>3400</v>
+        <v>2259</v>
       </c>
       <c r="R19" s="27" t="inlineStr">
         <is>
@@ -5465,7 +5465,7 @@
       </c>
       <c r="G7" s="34" t="inlineStr">
         <is>
-          <t>30/09/2026 13:16</t>
+          <t>30/09/2026 13:34</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="G15" s="34" t="inlineStr">
         <is>
-          <t>no_indicator</t>
+          <t>edu_disrupted_hazrds</t>
         </is>
       </c>
     </row>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="G26" s="34" t="inlineStr">
         <is>
-          <t>no_indicator</t>
+          <t>edu_disrupted_hazrds</t>
         </is>
       </c>
     </row>

</xml_diff>